<commit_message>
Update admin portal and Excel imports
</commit_message>
<xml_diff>
--- a/extracted_project_docs/ASRGH.COM/Excel template/members_import.xlsx
+++ b/extracted_project_docs/ASRGH.COM/Excel template/members_import.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SunGupta\Downloads\Website\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ASRGH_V2_NODE\ASRGH\ASRGH_V2_NODE\extracted_project_docs\ASRGH.COM\Excel template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{90FFB5D9-5F67-4A7A-924B-18B82F5D6D71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BD199B8-E909-4E49-9060-6165B4BDD085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DEF36577-7539-40EC-B015-596E2F5C3BAD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DEF36577-7539-40EC-B015-596E2F5C3BAD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,8 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -40,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="211">
   <si>
     <t>Column</t>
   </si>
@@ -217,47 +215,509 @@
     </r>
   </si>
   <si>
-    <t>MEM-0001</t>
-  </si>
-  <si>
-    <t>Rajesh</t>
-  </si>
-  <si>
-    <t>Sharma</t>
-  </si>
-  <si>
-    <t>Rajesh Sharma</t>
-  </si>
-  <si>
     <t>General</t>
   </si>
   <si>
-    <t>Member</t>
-  </si>
-  <si>
-    <t>President</t>
-  </si>
-  <si>
     <t>Active</t>
   </si>
   <si>
-    <t>MEM-0002</t>
-  </si>
-  <si>
-    <t>Amit</t>
-  </si>
-  <si>
-    <t>Verma</t>
-  </si>
-  <si>
-    <t>Amit Verma</t>
+    <t>EXCEL-UAT-001</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Date of Birth</t>
+  </si>
+  <si>
+    <t>15/08/1990</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Delhi</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Membership Status</t>
+  </si>
+  <si>
+    <t>Joined On</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Name 1</t>
+  </si>
+  <si>
+    <t>Middle 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last 1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address Line 1 </t>
+  </si>
+  <si>
+    <t>Rohini</t>
+  </si>
+  <si>
+    <t>Test notes</t>
+  </si>
+  <si>
+    <t>Name 2</t>
+  </si>
+  <si>
+    <t>Name 3</t>
+  </si>
+  <si>
+    <t>Name 4</t>
+  </si>
+  <si>
+    <t>Name 5</t>
+  </si>
+  <si>
+    <t>Name 6</t>
+  </si>
+  <si>
+    <t>Name 7</t>
+  </si>
+  <si>
+    <t>Name 8</t>
+  </si>
+  <si>
+    <t>Name 9</t>
+  </si>
+  <si>
+    <t>Name 10</t>
+  </si>
+  <si>
+    <t>Name 11</t>
+  </si>
+  <si>
+    <t>Name 12</t>
+  </si>
+  <si>
+    <t>Name 13</t>
+  </si>
+  <si>
+    <t>Name 14</t>
+  </si>
+  <si>
+    <t>Name 15</t>
+  </si>
+  <si>
+    <t>Name 16</t>
+  </si>
+  <si>
+    <t>Name 17</t>
+  </si>
+  <si>
+    <t>Name 18</t>
+  </si>
+  <si>
+    <t>Name 19</t>
+  </si>
+  <si>
+    <t>Middle 2</t>
+  </si>
+  <si>
+    <t>Middle 3</t>
+  </si>
+  <si>
+    <t>Middle 4</t>
+  </si>
+  <si>
+    <t>Middle 5</t>
+  </si>
+  <si>
+    <t>Middle 6</t>
+  </si>
+  <si>
+    <t>Middle 7</t>
+  </si>
+  <si>
+    <t>Middle 8</t>
+  </si>
+  <si>
+    <t>Middle 9</t>
+  </si>
+  <si>
+    <t>Middle 10</t>
+  </si>
+  <si>
+    <t>Middle 11</t>
+  </si>
+  <si>
+    <t>Middle 12</t>
+  </si>
+  <si>
+    <t>Middle 13</t>
+  </si>
+  <si>
+    <t>Middle 14</t>
+  </si>
+  <si>
+    <t>Middle 15</t>
+  </si>
+  <si>
+    <t>Middle 16</t>
+  </si>
+  <si>
+    <t>Middle 17</t>
+  </si>
+  <si>
+    <t>Middle 18</t>
+  </si>
+  <si>
+    <t>Middle 19</t>
+  </si>
+  <si>
+    <t>Last 2</t>
+  </si>
+  <si>
+    <t>Last 3</t>
+  </si>
+  <si>
+    <t>Last 4</t>
+  </si>
+  <si>
+    <t>Last 5</t>
+  </si>
+  <si>
+    <t>Last 6</t>
+  </si>
+  <si>
+    <t>Last 7</t>
+  </si>
+  <si>
+    <t>Last 8</t>
+  </si>
+  <si>
+    <t>Last 9</t>
+  </si>
+  <si>
+    <t>Last 10</t>
+  </si>
+  <si>
+    <t>Last 11</t>
+  </si>
+  <si>
+    <t>Last 12</t>
+  </si>
+  <si>
+    <t>Last 13</t>
+  </si>
+  <si>
+    <t>Last 14</t>
+  </si>
+  <si>
+    <t>Last 15</t>
+  </si>
+  <si>
+    <t>Last 16</t>
+  </si>
+  <si>
+    <t>Last 17</t>
+  </si>
+  <si>
+    <t>Last 18</t>
+  </si>
+  <si>
+    <t>Last 19</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-002</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-003</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-004</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-005</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-006</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-007</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-008</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-009</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-010</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-011</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-012</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-013</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-014</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-015</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-016</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-017</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-018</t>
+  </si>
+  <si>
+    <t>EXCEL-UAT-019</t>
+  </si>
+  <si>
+    <t>15/08/1991</t>
+  </si>
+  <si>
+    <t>15/08/1992</t>
+  </si>
+  <si>
+    <t>15/08/1993</t>
+  </si>
+  <si>
+    <t>15/08/1994</t>
+  </si>
+  <si>
+    <t>15/08/1995</t>
+  </si>
+  <si>
+    <t>15/08/1996</t>
+  </si>
+  <si>
+    <t>15/08/1997</t>
+  </si>
+  <si>
+    <t>15/08/1998</t>
+  </si>
+  <si>
+    <t>15/08/1999</t>
+  </si>
+  <si>
+    <t>15/08/2000</t>
+  </si>
+  <si>
+    <t>15/08/2001</t>
+  </si>
+  <si>
+    <t>15/08/2002</t>
+  </si>
+  <si>
+    <t>15/08/2003</t>
+  </si>
+  <si>
+    <t>15/08/2004</t>
+  </si>
+  <si>
+    <t>15/08/2005</t>
+  </si>
+  <si>
+    <t>15/08/2006</t>
+  </si>
+  <si>
+    <t>15/08/2007</t>
+  </si>
+  <si>
+    <t>15/08/2008</t>
+  </si>
+  <si>
+    <t>Address Line 3</t>
+  </si>
+  <si>
+    <t>Address Line 4</t>
+  </si>
+  <si>
+    <t>Address Line 5</t>
+  </si>
+  <si>
+    <t>Address Line 6</t>
+  </si>
+  <si>
+    <t>Address Line 7</t>
+  </si>
+  <si>
+    <t>Address Line 8</t>
+  </si>
+  <si>
+    <t>Address Line 9</t>
+  </si>
+  <si>
+    <t>Address Line 10</t>
+  </si>
+  <si>
+    <t>Address Line 11</t>
+  </si>
+  <si>
+    <t>Address Line 12</t>
+  </si>
+  <si>
+    <t>Address Line 13</t>
+  </si>
+  <si>
+    <t>Address Line 14</t>
+  </si>
+  <si>
+    <t>Address Line 15</t>
+  </si>
+  <si>
+    <t>Address Line 16</t>
+  </si>
+  <si>
+    <t>Address Line 17</t>
+  </si>
+  <si>
+    <t>Address Line 18</t>
+  </si>
+  <si>
+    <t>Address Line 19</t>
+  </si>
+  <si>
+    <t>Address Line 20</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com1</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com2</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com3</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com4</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com5</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com6</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com7</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com8</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com9</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com10</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com11</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com12</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com13</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com14</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com15</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com16</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com17</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com18</t>
+  </si>
+  <si>
+    <t>UatTest1@email.com19</t>
+  </si>
+  <si>
+    <t>Display 1</t>
+  </si>
+  <si>
+    <t>Display 2</t>
+  </si>
+  <si>
+    <t>Display 3</t>
+  </si>
+  <si>
+    <t>Display 4</t>
+  </si>
+  <si>
+    <t>Display 5</t>
+  </si>
+  <si>
+    <t>Display 6</t>
+  </si>
+  <si>
+    <t>Display 7</t>
+  </si>
+  <si>
+    <t>Display 8</t>
+  </si>
+  <si>
+    <t>Display 9</t>
+  </si>
+  <si>
+    <t>Display 10</t>
+  </si>
+  <si>
+    <t>Display 11</t>
+  </si>
+  <si>
+    <t>Display 12</t>
+  </si>
+  <si>
+    <t>Display 13</t>
+  </si>
+  <si>
+    <t>Display 14</t>
+  </si>
+  <si>
+    <t>Display 15</t>
+  </si>
+  <si>
+    <t>Display 16</t>
+  </si>
+  <si>
+    <t>Display 17</t>
+  </si>
+  <si>
+    <t>Display 18</t>
+  </si>
+  <si>
+    <t>Display 19</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -278,6 +738,20 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -296,10 +770,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -310,8 +785,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -644,95 +1123,1142 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21780322-E6DA-4786-8F50-A9335C6ED44B}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:S20"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="43.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:19" ht="28.8">
+      <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="28.8">
+      <c r="H1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="43.2">
       <c r="A2" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>9</v>
+        <v>192</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="28.8">
+        <v>45</v>
+      </c>
+      <c r="I2" s="2">
+        <v>999999999</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O2">
+        <v>110045</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="43.2">
       <c r="A3" s="2" t="s">
-        <v>53</v>
+        <v>119</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>55</v>
+        <v>83</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>49</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>50</v>
+        <v>137</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2" t="s">
-        <v>52</v>
+        <v>193</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3" s="2">
+        <v>1000000000</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O3">
+        <v>110046</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" ht="43.2">
+      <c r="A4" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I4" s="2">
+        <v>1000000001</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O4">
+        <v>110047</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="43.2">
+      <c r="A5" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I5" s="2">
+        <v>1000000002</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O5">
+        <v>110048</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="43.2">
+      <c r="A6" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I6" s="2">
+        <v>1000000003</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O6">
+        <v>110049</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="43.2">
+      <c r="A7" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I7" s="2">
+        <v>1000000004</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O7">
+        <v>110050</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="43.2">
+      <c r="A8" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I8" s="2">
+        <v>1000000005</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O8">
+        <v>110051</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S8" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="43.2">
+      <c r="A9" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" s="2">
+        <v>1000000006</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O9">
+        <v>110052</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S9" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="43.2">
+      <c r="A10" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I10" s="2">
+        <v>1000000007</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O10">
+        <v>110053</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S10" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="43.2">
+      <c r="A11" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I11" s="2">
+        <v>1000000008</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O11">
+        <v>110054</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S11" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="43.2">
+      <c r="A12" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I12" s="2">
+        <v>1000000009</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O12">
+        <v>110055</v>
+      </c>
+      <c r="P12" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q12" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S12" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="43.2">
+      <c r="A13" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I13" s="2">
+        <v>1000000010</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O13">
+        <v>110056</v>
+      </c>
+      <c r="P13" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q13" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S13" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="43.2">
+      <c r="A14" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I14" s="2">
+        <v>1000000011</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O14">
+        <v>110057</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q14" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S14" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" ht="43.2">
+      <c r="A15" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I15" s="2">
+        <v>1000000012</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O15">
+        <v>110058</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q15" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S15" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" ht="43.2">
+      <c r="A16" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I16" s="2">
+        <v>1000000013</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O16">
+        <v>110059</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q16" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S16" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" ht="43.2">
+      <c r="A17" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I17" s="2">
+        <v>1000000014</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O17">
+        <v>110060</v>
+      </c>
+      <c r="P17" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q17" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S17" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" ht="43.2">
+      <c r="A18" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I18" s="2">
+        <v>1000000015</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O18">
+        <v>110061</v>
+      </c>
+      <c r="P18" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q18" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S18" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" ht="43.2">
+      <c r="A19" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I19" s="2">
+        <v>1000000016</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N19" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O19">
+        <v>110062</v>
+      </c>
+      <c r="P19" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q19" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S19" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" ht="43.2">
+      <c r="A20" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I20" s="2">
+        <v>1000000017</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N20" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O20">
+        <v>110063</v>
+      </c>
+      <c r="P20" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q20" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S20" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="J2" r:id="rId1" xr:uid="{23D85521-4A74-4F5C-8BA8-4A743CF79549}"/>
+    <hyperlink ref="J3:J20" r:id="rId2" display="UatTest1@email.com1" xr:uid="{178755CE-4BDD-4FC5-BECE-1D6EB4DE6713}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>